<commit_message>
Adding Fam_Test_Automation repo on git
</commit_message>
<xml_diff>
--- a/Functional_Test_Cases.xlsx
+++ b/Functional_Test_Cases.xlsx
@@ -485,8 +485,8 @@
     <col width="23.90625" customWidth="1" style="1" min="4" max="4"/>
     <col width="24.81640625" customWidth="1" style="1" min="5" max="5"/>
     <col width="23.26953125" customWidth="1" style="1" min="6" max="6"/>
-    <col width="8.7265625" customWidth="1" style="1" min="7" max="9"/>
-    <col width="8.7265625" customWidth="1" style="1" min="10" max="16384"/>
+    <col width="8.7265625" customWidth="1" style="1" min="7" max="13"/>
+    <col width="8.7265625" customWidth="1" style="1" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,13 +527,13 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Step 1: [UI] Login to URL https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::: with credentials Username:ADMIN Password:admin123
+          <t xml:space="preserve">Step 1: Login to URL https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::: with credentials Username:ADMIN Password:admin123
 --ignore-https-errors
-Step 2. [UI] Go to Financial Management --&gt; Manage Documents
-Step 3. [UI] Filter Documents based on Transaction Type and Billing Period.
-Step 4. [UI] Select Transaction Type as Accruals and Billing Period as 01-Feb-2026 to 28-Feb-2026
-Step 5. [UI] Select the agreement RJILKO_AIRTTN_Exp from the display list and click on view document summary.
-Step 6. [UI] Capture the invoice details </t>
+Step 2. Go to Financial Management --&gt; Manage Documents
+Step 3. Filter Documents based on Transaction Type and Billing Period.
+Step 4. Select Transaction Type as Accruals and Billing Period as 01-Feb-2026 to 28-Feb-2026
+Step 5. Select the agreement RJILKO_AIRTTN_Exp from the display list and click on view document summary.
+Step 6. Capture the invoice details </t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Invoice captured for RJILDL_AIRTKN_ACTUAL_OFF_E_SO (Trans ID 6, INR, Tax 12,033.40)</t>
+          <t>Invoice captured for RJILDL_AIRTKN_ACTUAL_OFF_E_SO (Feb 2026 ACTUAL)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding input values for test cases
</commit_message>
<xml_diff>
--- a/Functional_Test_Cases.xlsx
+++ b/Functional_Test_Cases.xlsx
@@ -476,17 +476,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="23.7265625" customWidth="1" style="1" min="1" max="1"/>
     <col width="33.36328125" customWidth="1" style="1" min="2" max="2"/>
     <col width="68.08984375" customWidth="1" style="1" min="3" max="3"/>
-    <col width="23.90625" customWidth="1" style="1" min="4" max="4"/>
-    <col width="24.81640625" customWidth="1" style="1" min="5" max="5"/>
-    <col width="23.26953125" customWidth="1" style="1" min="6" max="6"/>
-    <col width="8.7265625" customWidth="1" style="1" min="7" max="13"/>
-    <col width="8.7265625" customWidth="1" style="1" min="14" max="16384"/>
+    <col width="40.26953125" customWidth="1" style="1" min="4" max="4"/>
+    <col width="23.90625" customWidth="1" style="1" min="5" max="5"/>
+    <col width="24.81640625" customWidth="1" style="1" min="6" max="6"/>
+    <col width="23.26953125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="8.7265625" customWidth="1" style="1" min="8" max="17"/>
+    <col width="8.7265625" customWidth="1" style="1" min="18" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,10 +508,15 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
+          <t>Input Values</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -527,23 +533,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Step 1: Login to URL https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::: with credentials Username:ADMIN Password:admin123
---ignore-https-errors
+          <t xml:space="preserve">Step 1: Login to {Application URL}: with credentials {Username} and {Password}
 Step 2. Go to Financial Management --&gt; Manage Documents
-Step 3. Filter Documents based on Transaction Type and Billing Period.
-Step 4. Select Transaction Type as Accruals and Billing Period as 01-Feb-2026 to 28-Feb-2026
-Step 5. Select the agreement RJILKO_AIRTTN_Exp from the display list and click on view document summary.
-Step 6. Capture the invoice details </t>
+Step 3. Filter Documents based on {Transaction Type} and {Billing Period}.
+Step 4. Select the {agreement} and display list and click on view document summary.
+Step 5. Capture the invoice details </t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Application URL -  https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::
+Username - ADMIN
+Password - admin123
+Transaction Type - Accruals
+Billing Period - 01-Feb-2026 to 28-Feb-2026
+Agreement - RJILKO_AIRTTN_Exp</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Invoice captured for RJILKO_AIRTTN_Exp (Feb 2026 ACCRUALS)</t>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>All steps completed; invoice details captured for RJILKO_AIRTTN_Exp</t>
         </is>
       </c>
     </row>
@@ -558,23 +572,31 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Step 1: Login to URL https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::: with credentials Username:ADMIN Password:admin123
---ignore-https-errors
+          <t xml:space="preserve">Step 1: Login to {Application URL}: with credentials {Username} and {Password}
 Step 2. Go to Financial Management --&gt; Manage Documents
-Step 3. Filter Documents based on Transaction Type and Billing Period.
-Step 4. Select Transaction Type as Actual and Billing Period as 01-Feb-2026 to 28-Feb-2026
-Step 5. Select the agreement RJILDL_AIRTKN_ACTUAL_OFF_E_SO from the display list and click on view document summary.
-Step 6. Capture the invoice details.</t>
+Step 3. Filter Documents based on {Transaction Type} and {Billing Period}.
+Step 4. Select the {agreement} and display list and click on view document summary.
+Step 5. Capture the invoice details </t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Application URL -  https://sg01dvxicta0003.csgidev.com:19100/ords/f?p=100:1:3135060356707::::
+Username - ADMIN
+Password - admin123
+Transaction Type - Actual
+Billing Period - 01-Feb-2026 to 28-Feb-2026
+Agreement - RJILDL_AIRTKN_ACTUAL_OFF_E_SO</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Invoice captured for RJILDL_AIRTKN_ACTUAL_OFF_E_SO (Feb 2026 ACTUAL)</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Invoice captured for RJILDL_AIRTKN_ACTUAL_OFF_E_SO (Trans ID 6, INR 12,033.40 total)</t>
         </is>
       </c>
     </row>
@@ -584,6 +606,7 @@
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -591,6 +614,7 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -598,6 +622,7 @@
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -605,6 +630,7 @@
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -612,6 +638,7 @@
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>